<commit_message>
EKA Kapı üstü dost proje kodu değiştrildi. ACM olan yer 000 olarak güncellendi.
</commit_message>
<xml_diff>
--- a/pages/gostergeler.xlsx
+++ b/pages/gostergeler.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work_Altium\GiTME\io_list\pages\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MTK\Butkon\Projeler\BTK42_EXCEL\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E72EBBE-01BF-451F-9FA2-442AF6E1A767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3518D69-7C3C-4CF3-B3CC-EAEA934CE4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -432,15 +432,9 @@
     <t>DP-EKA-DT-ACM-LOP-S2B1-01</t>
   </si>
   <si>
-    <t>DP-EKA-DT-ACM-LIP-S2B1-01</t>
-  </si>
-  <si>
     <t>https://github.com/btk42/DP-EKA-DT-ACM-LOP-S2B1-01</t>
   </si>
   <si>
-    <t>https://github.com/btk42/DP-EKA-DT-ACM-LIP-S2B1-01</t>
-  </si>
-  <si>
     <t>2x Dot</t>
   </si>
   <si>
@@ -475,6 +469,12 @@
   </si>
   <si>
     <t>https://github.com/btk42/DP-D19-3X-NUV-LOP-P2B1-01</t>
+  </si>
+  <si>
+    <t>DP-EKA-DT-000-LIP-S2B1-01</t>
+  </si>
+  <si>
+    <t>https://github.com/btk42/DP-EKA-DT-000-LIP-S2B1-01</t>
   </si>
 </sst>
 </file>
@@ -1467,7 +1467,7 @@
         <v>68</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L17" s="8"/>
     </row>
@@ -1476,7 +1476,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>69</v>
@@ -1503,7 +1503,7 @@
         <v>68</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="L18" s="8"/>
     </row>
@@ -1539,7 +1539,7 @@
         <v>68</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -1897,7 +1897,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>52</v>
@@ -1924,7 +1924,7 @@
         <v>68</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2317,7 +2317,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>32</v>
@@ -2344,7 +2344,7 @@
         <v>68</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2562,13 +2562,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E49" s="5" t="s">
         <v>48</v>
@@ -2589,7 +2589,7 @@
         <v>68</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2597,13 +2597,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E50" s="5" t="s">
         <v>48</v>
@@ -2624,7 +2624,7 @@
         <v>68</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.3">
@@ -2632,7 +2632,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>25</v>
@@ -2659,7 +2659,7 @@
         <v>68</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>